<commit_message>
working on Maas SeaBASS data
</commit_message>
<xml_diff>
--- a/CMAP_variableMetadata_additions.xlsx
+++ b/CMAP_variableMetadata_additions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\GitHub_niskin\BWrepos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82E17A3A-58D1-4E40-9607-AF0D4C6D4F64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3E3E7BC-8C06-419E-9468-1CB1DA88D69F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="45" yWindow="2205" windowWidth="27975" windowHeight="18135" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="465" yWindow="3720" windowWidth="25725" windowHeight="16245" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="notes" sheetId="4" r:id="rId1"/>
@@ -20,13 +20,14 @@
     <sheet name="964801_v1_pump_carbohydrates_bi" sheetId="8" r:id="rId5"/>
     <sheet name="964684_v1_amino_acids_biosscope" sheetId="9" r:id="rId6"/>
     <sheet name="920443_v1_biosscope_in_situ_pum" sheetId="10" r:id="rId7"/>
+    <sheet name="PVST_BATS_PLANKTON" sheetId="11" r:id="rId8"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1465" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1759" uniqueCount="467">
   <si>
     <t>Program</t>
   </si>
@@ -1217,6 +1218,216 @@
   </si>
   <si>
     <t>cells x 100 million per kg (cells*10^8/kg)</t>
+  </si>
+  <si>
+    <t>time</t>
+  </si>
+  <si>
+    <t>lat</t>
+  </si>
+  <si>
+    <t>lon</t>
+  </si>
+  <si>
+    <t>depth</t>
+  </si>
+  <si>
+    <t>hplc_gsfc_id</t>
+  </si>
+  <si>
+    <t>station</t>
+  </si>
+  <si>
+    <t>water_depth</t>
+  </si>
+  <si>
+    <t>bottle</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>volfilt</t>
+  </si>
+  <si>
+    <t>sample</t>
+  </si>
+  <si>
+    <t>allo</t>
+  </si>
+  <si>
+    <t>alpha-beta-car</t>
+  </si>
+  <si>
+    <t>but-fuco</t>
+  </si>
+  <si>
+    <t>chl_c1c2</t>
+  </si>
+  <si>
+    <t>chl_c3</t>
+  </si>
+  <si>
+    <t>chlide_a</t>
+  </si>
+  <si>
+    <t>diadino</t>
+  </si>
+  <si>
+    <t>diato</t>
+  </si>
+  <si>
+    <t>dp</t>
+  </si>
+  <si>
+    <t>dv_chl_a</t>
+  </si>
+  <si>
+    <t>dv_chl_b</t>
+  </si>
+  <si>
+    <t>fuco</t>
+  </si>
+  <si>
+    <t>gyro</t>
+  </si>
+  <si>
+    <t>hex-fuco</t>
+  </si>
+  <si>
+    <t>lut</t>
+  </si>
+  <si>
+    <t>mv_chl_a</t>
+  </si>
+  <si>
+    <t>mv_chl_b</t>
+  </si>
+  <si>
+    <t>neo</t>
+  </si>
+  <si>
+    <t>perid</t>
+  </si>
+  <si>
+    <t>phide_a</t>
+  </si>
+  <si>
+    <t>phytin_a</t>
+  </si>
+  <si>
+    <t>ppc</t>
+  </si>
+  <si>
+    <t>ppc_tcar</t>
+  </si>
+  <si>
+    <t>ppc_tpg</t>
+  </si>
+  <si>
+    <t>pras</t>
+  </si>
+  <si>
+    <t>psc</t>
+  </si>
+  <si>
+    <t>psc_tcar</t>
+  </si>
+  <si>
+    <t>psp</t>
+  </si>
+  <si>
+    <t>psp_tpg</t>
+  </si>
+  <si>
+    <t>tacc</t>
+  </si>
+  <si>
+    <t>tacc_tchla</t>
+  </si>
+  <si>
+    <t>tcar</t>
+  </si>
+  <si>
+    <t>tchl</t>
+  </si>
+  <si>
+    <t>tchl_tcar</t>
+  </si>
+  <si>
+    <t>tchla_tpg</t>
+  </si>
+  <si>
+    <t>tot_chl_a</t>
+  </si>
+  <si>
+    <t>tot_chl_b</t>
+  </si>
+  <si>
+    <t>tot_chl_c</t>
+  </si>
+  <si>
+    <t>tpg</t>
+  </si>
+  <si>
+    <t>viola</t>
+  </si>
+  <si>
+    <t>zea</t>
+  </si>
+  <si>
+    <t>filename</t>
+  </si>
+  <si>
+    <t>objectdetails</t>
+  </si>
+  <si>
+    <t>associated_files</t>
+  </si>
+  <si>
+    <t>associated_file_types</t>
+  </si>
+  <si>
+    <t>volume</t>
+  </si>
+  <si>
+    <t>data_provider_category_manual</t>
+  </si>
+  <si>
+    <t>scientificname_manual</t>
+  </si>
+  <si>
+    <t>scientificnameid_manual</t>
+  </si>
+  <si>
+    <t>area_cross_section</t>
+  </si>
+  <si>
+    <t>length_representation</t>
+  </si>
+  <si>
+    <t>width_representation</t>
+  </si>
+  <si>
+    <t>equivalent_spherical_diameter</t>
+  </si>
+  <si>
+    <t>volume_sampled_ml</t>
+  </si>
+  <si>
+    <t>volume_imaged_ml</t>
+  </si>
+  <si>
+    <t>volnet</t>
+  </si>
+  <si>
+    <t>splitfraction</t>
+  </si>
+  <si>
+    <t>particle_dilution_factor</t>
+  </si>
+  <si>
+    <t>biovolume</t>
   </si>
 </sst>
 </file>
@@ -7003,4 +7214,1052 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42F9E499-8F3B-4962-B041-C7E33D10A5CD}">
+  <dimension ref="A1:J72"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>397</v>
+      </c>
+      <c r="E2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F2" t="s">
+        <v>150</v>
+      </c>
+      <c r="G2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>398</v>
+      </c>
+      <c r="E3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G3" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>399</v>
+      </c>
+      <c r="E4" t="s">
+        <v>150</v>
+      </c>
+      <c r="F4" t="s">
+        <v>150</v>
+      </c>
+      <c r="G4" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>400</v>
+      </c>
+      <c r="E5" t="s">
+        <v>150</v>
+      </c>
+      <c r="F5" t="s">
+        <v>150</v>
+      </c>
+      <c r="G5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>401</v>
+      </c>
+      <c r="E6" t="s">
+        <v>150</v>
+      </c>
+      <c r="F6" t="s">
+        <v>150</v>
+      </c>
+      <c r="G6" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>402</v>
+      </c>
+      <c r="E7" t="s">
+        <v>150</v>
+      </c>
+      <c r="F7" t="s">
+        <v>150</v>
+      </c>
+      <c r="G7" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>403</v>
+      </c>
+      <c r="E8" t="s">
+        <v>150</v>
+      </c>
+      <c r="F8" t="s">
+        <v>150</v>
+      </c>
+      <c r="G8" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>404</v>
+      </c>
+      <c r="E9" t="s">
+        <v>150</v>
+      </c>
+      <c r="F9" t="s">
+        <v>150</v>
+      </c>
+      <c r="G9" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>405</v>
+      </c>
+      <c r="E10" t="s">
+        <v>150</v>
+      </c>
+      <c r="F10" t="s">
+        <v>150</v>
+      </c>
+      <c r="G10" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>397</v>
+      </c>
+      <c r="E11" t="s">
+        <v>150</v>
+      </c>
+      <c r="F11" t="s">
+        <v>150</v>
+      </c>
+      <c r="G11" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>406</v>
+      </c>
+      <c r="E12" t="s">
+        <v>150</v>
+      </c>
+      <c r="F12" t="s">
+        <v>150</v>
+      </c>
+      <c r="G12" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>407</v>
+      </c>
+      <c r="E13" t="s">
+        <v>150</v>
+      </c>
+      <c r="F13" t="s">
+        <v>150</v>
+      </c>
+      <c r="G13" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>408</v>
+      </c>
+      <c r="E14" t="s">
+        <v>150</v>
+      </c>
+      <c r="F14" t="s">
+        <v>150</v>
+      </c>
+      <c r="G14" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>409</v>
+      </c>
+      <c r="E15" t="s">
+        <v>150</v>
+      </c>
+      <c r="F15" t="s">
+        <v>150</v>
+      </c>
+      <c r="G15" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>410</v>
+      </c>
+      <c r="E16" t="s">
+        <v>150</v>
+      </c>
+      <c r="F16" t="s">
+        <v>150</v>
+      </c>
+      <c r="G16" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>411</v>
+      </c>
+      <c r="E17" t="s">
+        <v>150</v>
+      </c>
+      <c r="F17" t="s">
+        <v>150</v>
+      </c>
+      <c r="G17" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>412</v>
+      </c>
+      <c r="E18" t="s">
+        <v>150</v>
+      </c>
+      <c r="F18" t="s">
+        <v>150</v>
+      </c>
+      <c r="G18" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>413</v>
+      </c>
+      <c r="E19" t="s">
+        <v>150</v>
+      </c>
+      <c r="F19" t="s">
+        <v>150</v>
+      </c>
+      <c r="G19" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>414</v>
+      </c>
+      <c r="E20" t="s">
+        <v>150</v>
+      </c>
+      <c r="F20" t="s">
+        <v>150</v>
+      </c>
+      <c r="G20" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>415</v>
+      </c>
+      <c r="E21" t="s">
+        <v>150</v>
+      </c>
+      <c r="F21" t="s">
+        <v>150</v>
+      </c>
+      <c r="G21" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>416</v>
+      </c>
+      <c r="E22" t="s">
+        <v>150</v>
+      </c>
+      <c r="F22" t="s">
+        <v>150</v>
+      </c>
+      <c r="G22" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>417</v>
+      </c>
+      <c r="E23" t="s">
+        <v>150</v>
+      </c>
+      <c r="F23" t="s">
+        <v>150</v>
+      </c>
+      <c r="G23" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>418</v>
+      </c>
+      <c r="E24" t="s">
+        <v>150</v>
+      </c>
+      <c r="F24" t="s">
+        <v>150</v>
+      </c>
+      <c r="G24" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>419</v>
+      </c>
+      <c r="E25" t="s">
+        <v>150</v>
+      </c>
+      <c r="F25" t="s">
+        <v>150</v>
+      </c>
+      <c r="G25" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>420</v>
+      </c>
+      <c r="E26" t="s">
+        <v>150</v>
+      </c>
+      <c r="F26" t="s">
+        <v>150</v>
+      </c>
+      <c r="G26" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>421</v>
+      </c>
+      <c r="E27" t="s">
+        <v>150</v>
+      </c>
+      <c r="F27" t="s">
+        <v>150</v>
+      </c>
+      <c r="G27" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>422</v>
+      </c>
+      <c r="E28" t="s">
+        <v>150</v>
+      </c>
+      <c r="F28" t="s">
+        <v>150</v>
+      </c>
+      <c r="G28" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>423</v>
+      </c>
+      <c r="E29" t="s">
+        <v>150</v>
+      </c>
+      <c r="F29" t="s">
+        <v>150</v>
+      </c>
+      <c r="G29" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>424</v>
+      </c>
+      <c r="E30" t="s">
+        <v>150</v>
+      </c>
+      <c r="F30" t="s">
+        <v>150</v>
+      </c>
+      <c r="G30" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>425</v>
+      </c>
+      <c r="E31" t="s">
+        <v>150</v>
+      </c>
+      <c r="F31" t="s">
+        <v>150</v>
+      </c>
+      <c r="G31" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>426</v>
+      </c>
+      <c r="E32" t="s">
+        <v>150</v>
+      </c>
+      <c r="F32" t="s">
+        <v>150</v>
+      </c>
+      <c r="G32" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>427</v>
+      </c>
+      <c r="E33" t="s">
+        <v>150</v>
+      </c>
+      <c r="F33" t="s">
+        <v>150</v>
+      </c>
+      <c r="G33" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>428</v>
+      </c>
+      <c r="E34" t="s">
+        <v>150</v>
+      </c>
+      <c r="F34" t="s">
+        <v>150</v>
+      </c>
+      <c r="G34" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>429</v>
+      </c>
+      <c r="E35" t="s">
+        <v>150</v>
+      </c>
+      <c r="F35" t="s">
+        <v>150</v>
+      </c>
+      <c r="G35" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>430</v>
+      </c>
+      <c r="E36" t="s">
+        <v>150</v>
+      </c>
+      <c r="F36" t="s">
+        <v>150</v>
+      </c>
+      <c r="G36" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>431</v>
+      </c>
+      <c r="E37" t="s">
+        <v>150</v>
+      </c>
+      <c r="F37" t="s">
+        <v>150</v>
+      </c>
+      <c r="G37" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>432</v>
+      </c>
+      <c r="E38" t="s">
+        <v>150</v>
+      </c>
+      <c r="F38" t="s">
+        <v>150</v>
+      </c>
+      <c r="G38" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>433</v>
+      </c>
+      <c r="E39" t="s">
+        <v>150</v>
+      </c>
+      <c r="F39" t="s">
+        <v>150</v>
+      </c>
+      <c r="G39" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>434</v>
+      </c>
+      <c r="E40" t="s">
+        <v>150</v>
+      </c>
+      <c r="F40" t="s">
+        <v>150</v>
+      </c>
+      <c r="G40" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>435</v>
+      </c>
+      <c r="E41" t="s">
+        <v>150</v>
+      </c>
+      <c r="F41" t="s">
+        <v>150</v>
+      </c>
+      <c r="G41" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>436</v>
+      </c>
+      <c r="E42" t="s">
+        <v>150</v>
+      </c>
+      <c r="F42" t="s">
+        <v>150</v>
+      </c>
+      <c r="G42" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>437</v>
+      </c>
+      <c r="E43" t="s">
+        <v>150</v>
+      </c>
+      <c r="F43" t="s">
+        <v>150</v>
+      </c>
+      <c r="G43" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>438</v>
+      </c>
+      <c r="E44" t="s">
+        <v>150</v>
+      </c>
+      <c r="F44" t="s">
+        <v>150</v>
+      </c>
+      <c r="G44" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>439</v>
+      </c>
+      <c r="E45" t="s">
+        <v>150</v>
+      </c>
+      <c r="F45" t="s">
+        <v>150</v>
+      </c>
+      <c r="G45" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>440</v>
+      </c>
+      <c r="E46" t="s">
+        <v>150</v>
+      </c>
+      <c r="F46" t="s">
+        <v>150</v>
+      </c>
+      <c r="G46" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>441</v>
+      </c>
+      <c r="E47" t="s">
+        <v>150</v>
+      </c>
+      <c r="F47" t="s">
+        <v>150</v>
+      </c>
+      <c r="G47" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>442</v>
+      </c>
+      <c r="E48" t="s">
+        <v>150</v>
+      </c>
+      <c r="F48" t="s">
+        <v>150</v>
+      </c>
+      <c r="G48" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>443</v>
+      </c>
+      <c r="E49" t="s">
+        <v>150</v>
+      </c>
+      <c r="F49" t="s">
+        <v>150</v>
+      </c>
+      <c r="G49" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>444</v>
+      </c>
+      <c r="E50" t="s">
+        <v>150</v>
+      </c>
+      <c r="F50" t="s">
+        <v>150</v>
+      </c>
+      <c r="G50" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>445</v>
+      </c>
+      <c r="E51" t="s">
+        <v>150</v>
+      </c>
+      <c r="F51" t="s">
+        <v>150</v>
+      </c>
+      <c r="G51" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>446</v>
+      </c>
+      <c r="E52" t="s">
+        <v>150</v>
+      </c>
+      <c r="F52" t="s">
+        <v>150</v>
+      </c>
+      <c r="G52" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>447</v>
+      </c>
+      <c r="E53" t="s">
+        <v>150</v>
+      </c>
+      <c r="F53" t="s">
+        <v>150</v>
+      </c>
+      <c r="G53" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>448</v>
+      </c>
+      <c r="E54" t="s">
+        <v>150</v>
+      </c>
+      <c r="F54" t="s">
+        <v>150</v>
+      </c>
+      <c r="G54" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>449</v>
+      </c>
+      <c r="E55" t="s">
+        <v>150</v>
+      </c>
+      <c r="F55" t="s">
+        <v>150</v>
+      </c>
+      <c r="G55" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>450</v>
+      </c>
+      <c r="E56" t="s">
+        <v>150</v>
+      </c>
+      <c r="F56" t="s">
+        <v>150</v>
+      </c>
+      <c r="G56" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>451</v>
+      </c>
+      <c r="E57" t="s">
+        <v>150</v>
+      </c>
+      <c r="F57" t="s">
+        <v>150</v>
+      </c>
+      <c r="G57" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>452</v>
+      </c>
+      <c r="E58" t="s">
+        <v>150</v>
+      </c>
+      <c r="F58" t="s">
+        <v>150</v>
+      </c>
+      <c r="G58" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>453</v>
+      </c>
+      <c r="E59" t="s">
+        <v>150</v>
+      </c>
+      <c r="F59" t="s">
+        <v>150</v>
+      </c>
+      <c r="G59" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>454</v>
+      </c>
+      <c r="E60" t="s">
+        <v>150</v>
+      </c>
+      <c r="F60" t="s">
+        <v>150</v>
+      </c>
+      <c r="G60" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>455</v>
+      </c>
+      <c r="E61" t="s">
+        <v>150</v>
+      </c>
+      <c r="F61" t="s">
+        <v>150</v>
+      </c>
+      <c r="G61" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>456</v>
+      </c>
+      <c r="E62" t="s">
+        <v>150</v>
+      </c>
+      <c r="F62" t="s">
+        <v>150</v>
+      </c>
+      <c r="G62" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>457</v>
+      </c>
+      <c r="E63" t="s">
+        <v>150</v>
+      </c>
+      <c r="F63" t="s">
+        <v>150</v>
+      </c>
+      <c r="G63" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>458</v>
+      </c>
+      <c r="E64" t="s">
+        <v>150</v>
+      </c>
+      <c r="F64" t="s">
+        <v>150</v>
+      </c>
+      <c r="G64" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>459</v>
+      </c>
+      <c r="E65" t="s">
+        <v>150</v>
+      </c>
+      <c r="F65" t="s">
+        <v>150</v>
+      </c>
+      <c r="G65" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>460</v>
+      </c>
+      <c r="E66" t="s">
+        <v>150</v>
+      </c>
+      <c r="F66" t="s">
+        <v>150</v>
+      </c>
+      <c r="G66" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>461</v>
+      </c>
+      <c r="E67" t="s">
+        <v>150</v>
+      </c>
+      <c r="F67" t="s">
+        <v>150</v>
+      </c>
+      <c r="G67" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>462</v>
+      </c>
+      <c r="E68" t="s">
+        <v>150</v>
+      </c>
+      <c r="F68" t="s">
+        <v>150</v>
+      </c>
+      <c r="G68" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>463</v>
+      </c>
+      <c r="E69" t="s">
+        <v>150</v>
+      </c>
+      <c r="F69" t="s">
+        <v>150</v>
+      </c>
+      <c r="G69" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>464</v>
+      </c>
+      <c r="E70" t="s">
+        <v>150</v>
+      </c>
+      <c r="F70" t="s">
+        <v>150</v>
+      </c>
+      <c r="G70" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>465</v>
+      </c>
+      <c r="E71" t="s">
+        <v>150</v>
+      </c>
+      <c r="F71" t="s">
+        <v>150</v>
+      </c>
+      <c r="G71" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>466</v>
+      </c>
+      <c r="E72" t="s">
+        <v>150</v>
+      </c>
+      <c r="F72" t="s">
+        <v>150</v>
+      </c>
+      <c r="G72" t="s">
+        <v>197</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
wrapping up for day on SeaBASS but need input from AM and LBB
</commit_message>
<xml_diff>
--- a/CMAP_variableMetadata_additions.xlsx
+++ b/CMAP_variableMetadata_additions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\GitHub_niskin\BWrepos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3E3E7BC-8C06-419E-9468-1CB1DA88D69F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E14BE72-E1C8-4D5F-B170-33F1AF2DC8A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="465" yWindow="3720" windowWidth="25725" windowHeight="16245" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="270" yWindow="165" windowWidth="35295" windowHeight="18930" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="notes" sheetId="4" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1759" uniqueCount="467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1961" uniqueCount="542">
   <si>
     <t>Program</t>
   </si>
@@ -1223,160 +1223,331 @@
     <t>time</t>
   </si>
   <si>
+    <t>Sample time [GMT]</t>
+  </si>
+  <si>
+    <t>hh:mm:ss</t>
+  </si>
+  <si>
+    <t>BIOS-SCOPE, BIOS, Simons Foundation International, bio, biogeo, biogeochemistry, biology, flowCAM, Zooscan, net tows, Discrete, Bottle, cruise, Discrete, in situ, insitu, in-situ, North Atlantic Ocean, observation</t>
+  </si>
+  <si>
     <t>lat</t>
   </si>
   <si>
+    <t>Sample latitude (decimal fractions; -90 to 90)</t>
+  </si>
+  <si>
+    <t>degrees</t>
+  </si>
+  <si>
     <t>lon</t>
   </si>
   <si>
+    <t>Sample longitude (decimal fractions; -180 to 180)</t>
+  </si>
+  <si>
     <t>depth</t>
   </si>
   <si>
+    <t>Depth of measurement</t>
+  </si>
+  <si>
     <t>hplc_gsfc_id</t>
   </si>
   <si>
+    <t>NASA GSFC HPLC processing idenfication number (i.e. 'GSFC HPLC lab sampler code')</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
     <t>station</t>
   </si>
   <si>
+    <t>Sample station</t>
+  </si>
+  <si>
     <t>water_depth</t>
   </si>
   <si>
+    <t>The water (bottom) depth where the data were collected</t>
+  </si>
+  <si>
     <t>bottle</t>
   </si>
   <si>
+    <t>Number used to identify a specific bottle within an array of bottle samples collected</t>
+  </si>
+  <si>
     <t>date</t>
   </si>
   <si>
+    <t>Sample date</t>
+  </si>
+  <si>
+    <t>yyyymmdd</t>
+  </si>
+  <si>
     <t>volfilt</t>
   </si>
   <si>
+    <t>L</t>
+  </si>
+  <si>
     <t>sample</t>
   </si>
   <si>
+    <t>Sample number</t>
+  </si>
+  <si>
     <t>allo</t>
   </si>
   <si>
+    <t>HPLC Alloxanthin</t>
+  </si>
+  <si>
+    <t>mg/m^3</t>
+  </si>
+  <si>
     <t>alpha-beta-car</t>
   </si>
   <si>
+    <t>HPLC Alpha (Beta,epsilon) + Beta (Beta,beta) Carotenes</t>
+  </si>
+  <si>
     <t>but-fuco</t>
   </si>
   <si>
+    <t>HPLC 19'-Butanoyloxyfucoxanthin</t>
+  </si>
+  <si>
     <t>chl_c1c2</t>
   </si>
   <si>
+    <t>HPLC Chlorophyll c1 + c2 + Mg_DVP</t>
+  </si>
+  <si>
     <t>chl_c3</t>
   </si>
   <si>
+    <t>HPLC Chlorophyll c3</t>
+  </si>
+  <si>
     <t>chlide_a</t>
   </si>
   <si>
+    <t>HPLC Chlorophyllide a</t>
+  </si>
+  <si>
     <t>diadino</t>
   </si>
   <si>
+    <t>HPLC Diadinoxanthin</t>
+  </si>
+  <si>
     <t>diato</t>
   </si>
   <si>
+    <t>HPLC Diatoxanthin</t>
+  </si>
+  <si>
     <t>dp</t>
   </si>
   <si>
+    <t>Total diagnostic pigments (PSC + Allo + Zea + Tot_Chl_b)</t>
+  </si>
+  <si>
     <t>dv_chl_a</t>
   </si>
   <si>
+    <t>HPLC Divinyl Chorophyll a</t>
+  </si>
+  <si>
     <t>dv_chl_b</t>
   </si>
   <si>
+    <t>HPLC Divinyl Chorophyll b</t>
+  </si>
+  <si>
     <t>fuco</t>
   </si>
   <si>
+    <t>HPLC Fucoxanthin</t>
+  </si>
+  <si>
     <t>gyro</t>
   </si>
   <si>
+    <t>HPLC Gyroxanthin-Diester</t>
+  </si>
+  <si>
     <t>hex-fuco</t>
   </si>
   <si>
+    <t>HPLC 19'-Hexanoyloxyfucoxanthin</t>
+  </si>
+  <si>
     <t>lut</t>
   </si>
   <si>
+    <t>HPLC Lutein</t>
+  </si>
+  <si>
     <t>mv_chl_a</t>
   </si>
   <si>
+    <t>HPLC Monovinyl Chorophyll a</t>
+  </si>
+  <si>
     <t>mv_chl_b</t>
   </si>
   <si>
+    <t>HPLC Monovinyl Chorophyll b</t>
+  </si>
+  <si>
     <t>neo</t>
   </si>
   <si>
+    <t>HPLC Neoxanthin</t>
+  </si>
+  <si>
     <t>perid</t>
   </si>
   <si>
+    <t>HPLC Peridinin</t>
+  </si>
+  <si>
     <t>phide_a</t>
   </si>
   <si>
+    <t>HPLC Pheophorbide a</t>
+  </si>
+  <si>
     <t>phytin_a</t>
   </si>
   <si>
+    <t>HPLC Pheophytin a</t>
+  </si>
+  <si>
     <t>ppc</t>
   </si>
   <si>
+    <t>Photoprotective carotenoids (Allo + Diadino + Diato + Zeo + alpha-beta-Car)</t>
+  </si>
+  <si>
     <t>ppc_tcar</t>
   </si>
   <si>
+    <t>Ratio of PPC to Tcar</t>
+  </si>
+  <si>
     <t>ppc_tpg</t>
   </si>
   <si>
+    <t>Ratio of PPC to Tpg</t>
+  </si>
+  <si>
     <t>pras</t>
   </si>
   <si>
+    <t>HPLC Prasinoxanthin</t>
+  </si>
+  <si>
     <t>psc</t>
   </si>
   <si>
+    <t>Photosynthetic carotenoids (But-fuco + Fuco + Hex-fuco + Perid)</t>
+  </si>
+  <si>
     <t>psc_tcar</t>
   </si>
   <si>
+    <t>Ratio of PSC to Tcar</t>
+  </si>
+  <si>
     <t>psp</t>
   </si>
   <si>
+    <t>Photosynthetic pigments (PSC + Tchl)</t>
+  </si>
+  <si>
     <t>psp_tpg</t>
   </si>
   <si>
+    <t>Ratio of PSP to Tpg</t>
+  </si>
+  <si>
     <t>tacc</t>
   </si>
   <si>
+    <t>Total accessory pigments (PPC + PSC + Tot_Chl_b + Tot_Chl_c)</t>
+  </si>
+  <si>
     <t>tacc_tchla</t>
   </si>
   <si>
+    <t>Ratio of Tacc to Tot_Chl_a</t>
+  </si>
+  <si>
     <t>tcar</t>
   </si>
   <si>
+    <t>Total carotenoids (PPC + PSC)</t>
+  </si>
+  <si>
     <t>tchl</t>
   </si>
   <si>
+    <t>Tot_Chl_a + Tot_Chl_b + Tot_Chl_c</t>
+  </si>
+  <si>
     <t>tchl_tcar</t>
   </si>
   <si>
+    <t>Ratio of Tchl to Tcar</t>
+  </si>
+  <si>
     <t>tchla_tpg</t>
   </si>
   <si>
+    <t>Ratio of Tot_chl_a to Tpg</t>
+  </si>
+  <si>
     <t>tot_chl_a</t>
   </si>
   <si>
+    <t>HPLC DV_Chl_a + MV_Chl_a + Chlide_a + Chl_a_allom + Chl_a_prime</t>
+  </si>
+  <si>
     <t>tot_chl_b</t>
   </si>
   <si>
+    <t>HPLC DV_Chl_b + MV_Chl_b</t>
+  </si>
+  <si>
     <t>tot_chl_c</t>
   </si>
   <si>
+    <t>HPLC chl_c1 + chl_c2 (i.e., chl_c1c2) + chl_c3</t>
+  </si>
+  <si>
     <t>tpg</t>
   </si>
   <si>
+    <t>Total pigment concentration</t>
+  </si>
+  <si>
     <t>viola</t>
   </si>
   <si>
+    <t>HPLC Violaxanthin</t>
+  </si>
+  <si>
     <t>zea</t>
   </si>
   <si>
-    <t>filename</t>
+    <t>HPLC Zeaxanthin</t>
   </si>
   <si>
     <t>objectdetails</t>
@@ -1391,21 +1562,36 @@
     <t>volume</t>
   </si>
   <si>
+    <t>Volume used in experiment</t>
+  </si>
+  <si>
     <t>data_provider_category_manual</t>
   </si>
   <si>
+    <t>A category used by the data provider to name the organism or particle for a manual identification, not necessarily a scientific name.</t>
+  </si>
+  <si>
     <t>scientificname_manual</t>
   </si>
   <si>
+    <t>A scientific name from a recognized taxonomic reference database (e.g., World Register of Marine Species, AlgaeBase) at the lowest level that matches the data provider's category, for a manual identification matched to scientificNameID. Generally, the ROI corresponds to an occurrence assigned to a single taxonomic name.</t>
+  </si>
+  <si>
     <t>scientificnameid_manual</t>
   </si>
   <si>
     <t>area_cross_section</t>
   </si>
   <si>
+    <t>um^2</t>
+  </si>
+  <si>
     <t>length_representation</t>
   </si>
   <si>
+    <t>um</t>
+  </si>
+  <si>
     <t>width_representation</t>
   </si>
   <si>
@@ -1415,9 +1601,18 @@
     <t>volume_sampled_ml</t>
   </si>
   <si>
+    <t>Volume sample by flow cytometer in milliliters</t>
+  </si>
+  <si>
+    <t>mL</t>
+  </si>
+  <si>
     <t>volume_imaged_ml</t>
   </si>
   <si>
+    <t>Volume imaged by imaging flow cytometer in milliliters</t>
+  </si>
+  <si>
     <t>volnet</t>
   </si>
   <si>
@@ -1428,6 +1623,36 @@
   </si>
   <si>
     <t>biovolume</t>
+  </si>
+  <si>
+    <t>Biovolume for the target detected within the ROI determined by means specified in the biovolume calculation method or protocol document.</t>
+  </si>
+  <si>
+    <t>um^3</t>
+  </si>
+  <si>
+    <t>File type of an associated file.</t>
+  </si>
+  <si>
+    <t>the number of the image in EcoTaxa which is found as follows:  https://ecotaxa.obs-vlfr.fr/objectdetails/ &amp; objid (objid = the number of the image in EcoTaxa)</t>
+  </si>
+  <si>
+    <t>object_length, in um, major; Representation of length of the target detected within the ROI or largest mesh size for which the target could be retained, determined by means specified in the image processing method or protocol document.</t>
+  </si>
+  <si>
+    <t>object_width, in um, minor; Representation of width of the target detected within the ROI or smallest mesh size through which the target could pass, determined by means specified in the image processing method or protocol document.</t>
+  </si>
+  <si>
+    <t>object_diameter_esd ; Equivalent spherical diameter of the target detected within the ROI determined by means specified in the image processing method or protocol document.</t>
+  </si>
+  <si>
+    <t>File name of an associated file</t>
+  </si>
+  <si>
+    <t>object_area_filled; Cross-sectional area of the target detected within the ROI determined by means specified in the image processing method or protocol document.</t>
+  </si>
+  <si>
+    <t>only net samples?</t>
   </si>
 </sst>
 </file>
@@ -1458,12 +1683,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -1494,13 +1731,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7218,13 +7458,13 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42F9E499-8F3B-4962-B041-C7E33D10A5CD}">
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="171.5703125" customWidth="1"/>
     <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.5703125" customWidth="1"/>
     <col min="5" max="5" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -7269,6 +7509,12 @@
       <c r="A2" t="s">
         <v>397</v>
       </c>
+      <c r="B2" t="s">
+        <v>398</v>
+      </c>
+      <c r="D2" t="s">
+        <v>399</v>
+      </c>
       <c r="E2" t="s">
         <v>150</v>
       </c>
@@ -7278,10 +7524,22 @@
       <c r="G2" t="s">
         <v>197</v>
       </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>398</v>
+        <v>401</v>
+      </c>
+      <c r="B3" t="s">
+        <v>402</v>
+      </c>
+      <c r="D3" t="s">
+        <v>403</v>
       </c>
       <c r="E3" t="s">
         <v>150</v>
@@ -7292,10 +7550,22 @@
       <c r="G3" t="s">
         <v>197</v>
       </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>399</v>
+        <v>404</v>
+      </c>
+      <c r="B4" t="s">
+        <v>405</v>
+      </c>
+      <c r="D4" t="s">
+        <v>403</v>
       </c>
       <c r="E4" t="s">
         <v>150</v>
@@ -7306,10 +7576,22 @@
       <c r="G4" t="s">
         <v>197</v>
       </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>400</v>
+        <v>406</v>
+      </c>
+      <c r="B5" t="s">
+        <v>407</v>
+      </c>
+      <c r="D5" t="s">
+        <v>192</v>
       </c>
       <c r="E5" t="s">
         <v>150</v>
@@ -7320,10 +7602,22 @@
       <c r="G5" t="s">
         <v>197</v>
       </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>401</v>
+        <v>408</v>
+      </c>
+      <c r="B6" t="s">
+        <v>409</v>
+      </c>
+      <c r="D6" t="s">
+        <v>410</v>
       </c>
       <c r="E6" t="s">
         <v>150</v>
@@ -7334,10 +7628,22 @@
       <c r="G6" t="s">
         <v>197</v>
       </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>402</v>
+        <v>411</v>
+      </c>
+      <c r="B7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D7" t="s">
+        <v>410</v>
       </c>
       <c r="E7" t="s">
         <v>150</v>
@@ -7348,10 +7654,22 @@
       <c r="G7" t="s">
         <v>197</v>
       </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>403</v>
+        <v>413</v>
+      </c>
+      <c r="B8" t="s">
+        <v>414</v>
+      </c>
+      <c r="D8" t="s">
+        <v>192</v>
       </c>
       <c r="E8" t="s">
         <v>150</v>
@@ -7362,10 +7680,22 @@
       <c r="G8" t="s">
         <v>197</v>
       </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>404</v>
+        <v>415</v>
+      </c>
+      <c r="B9" t="s">
+        <v>416</v>
+      </c>
+      <c r="D9" t="s">
+        <v>410</v>
       </c>
       <c r="E9" t="s">
         <v>150</v>
@@ -7376,10 +7706,22 @@
       <c r="G9" t="s">
         <v>197</v>
       </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>405</v>
+        <v>417</v>
+      </c>
+      <c r="B10" t="s">
+        <v>418</v>
+      </c>
+      <c r="D10" t="s">
+        <v>419</v>
       </c>
       <c r="E10" t="s">
         <v>150</v>
@@ -7389,12 +7731,24 @@
       </c>
       <c r="G10" t="s">
         <v>197</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10" t="s">
+        <v>400</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>397</v>
       </c>
+      <c r="B11" t="s">
+        <v>398</v>
+      </c>
+      <c r="D11" t="s">
+        <v>399</v>
+      </c>
       <c r="E11" t="s">
         <v>150</v>
       </c>
@@ -7404,10 +7758,22 @@
       <c r="G11" t="s">
         <v>197</v>
       </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>406</v>
+        <v>420</v>
+      </c>
+      <c r="B12" t="s">
+        <v>211</v>
+      </c>
+      <c r="D12" t="s">
+        <v>421</v>
       </c>
       <c r="E12" t="s">
         <v>150</v>
@@ -7418,10 +7784,22 @@
       <c r="G12" t="s">
         <v>197</v>
       </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>407</v>
+        <v>422</v>
+      </c>
+      <c r="B13" t="s">
+        <v>423</v>
+      </c>
+      <c r="D13" t="s">
+        <v>410</v>
       </c>
       <c r="E13" t="s">
         <v>150</v>
@@ -7432,10 +7810,22 @@
       <c r="G13" t="s">
         <v>197</v>
       </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>408</v>
+        <v>424</v>
+      </c>
+      <c r="B14" t="s">
+        <v>425</v>
+      </c>
+      <c r="D14" t="s">
+        <v>426</v>
       </c>
       <c r="E14" t="s">
         <v>150</v>
@@ -7446,10 +7836,22 @@
       <c r="G14" t="s">
         <v>197</v>
       </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+      <c r="I14" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>409</v>
+        <v>427</v>
+      </c>
+      <c r="B15" t="s">
+        <v>428</v>
+      </c>
+      <c r="D15" t="s">
+        <v>426</v>
       </c>
       <c r="E15" t="s">
         <v>150</v>
@@ -7460,10 +7862,22 @@
       <c r="G15" t="s">
         <v>197</v>
       </c>
+      <c r="H15">
+        <v>1</v>
+      </c>
+      <c r="I15" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>410</v>
+        <v>429</v>
+      </c>
+      <c r="B16" t="s">
+        <v>430</v>
+      </c>
+      <c r="D16" t="s">
+        <v>426</v>
       </c>
       <c r="E16" t="s">
         <v>150</v>
@@ -7474,10 +7888,22 @@
       <c r="G16" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H16">
+        <v>1</v>
+      </c>
+      <c r="I16" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>411</v>
+        <v>431</v>
+      </c>
+      <c r="B17" t="s">
+        <v>432</v>
+      </c>
+      <c r="D17" t="s">
+        <v>426</v>
       </c>
       <c r="E17" t="s">
         <v>150</v>
@@ -7488,10 +7914,22 @@
       <c r="G17" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H17">
+        <v>1</v>
+      </c>
+      <c r="I17" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>412</v>
+        <v>433</v>
+      </c>
+      <c r="B18" t="s">
+        <v>434</v>
+      </c>
+      <c r="D18" t="s">
+        <v>426</v>
       </c>
       <c r="E18" t="s">
         <v>150</v>
@@ -7502,10 +7940,22 @@
       <c r="G18" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H18">
+        <v>1</v>
+      </c>
+      <c r="I18" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>413</v>
+        <v>435</v>
+      </c>
+      <c r="B19" t="s">
+        <v>436</v>
+      </c>
+      <c r="D19" t="s">
+        <v>426</v>
       </c>
       <c r="E19" t="s">
         <v>150</v>
@@ -7516,10 +7966,22 @@
       <c r="G19" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H19">
+        <v>1</v>
+      </c>
+      <c r="I19" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>414</v>
+        <v>437</v>
+      </c>
+      <c r="B20" t="s">
+        <v>438</v>
+      </c>
+      <c r="D20" t="s">
+        <v>426</v>
       </c>
       <c r="E20" t="s">
         <v>150</v>
@@ -7530,10 +7992,22 @@
       <c r="G20" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H20">
+        <v>1</v>
+      </c>
+      <c r="I20" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>415</v>
+        <v>439</v>
+      </c>
+      <c r="B21" t="s">
+        <v>440</v>
+      </c>
+      <c r="D21" t="s">
+        <v>426</v>
       </c>
       <c r="E21" t="s">
         <v>150</v>
@@ -7544,10 +8018,22 @@
       <c r="G21" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H21">
+        <v>1</v>
+      </c>
+      <c r="I21" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>416</v>
+        <v>441</v>
+      </c>
+      <c r="B22" t="s">
+        <v>442</v>
+      </c>
+      <c r="D22" t="s">
+        <v>426</v>
       </c>
       <c r="E22" t="s">
         <v>150</v>
@@ -7558,10 +8044,22 @@
       <c r="G22" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H22">
+        <v>1</v>
+      </c>
+      <c r="I22" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>417</v>
+        <v>443</v>
+      </c>
+      <c r="B23" t="s">
+        <v>444</v>
+      </c>
+      <c r="D23" t="s">
+        <v>426</v>
       </c>
       <c r="E23" t="s">
         <v>150</v>
@@ -7572,10 +8070,22 @@
       <c r="G23" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H23">
+        <v>1</v>
+      </c>
+      <c r="I23" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>418</v>
+        <v>445</v>
+      </c>
+      <c r="B24" t="s">
+        <v>446</v>
+      </c>
+      <c r="D24" t="s">
+        <v>426</v>
       </c>
       <c r="E24" t="s">
         <v>150</v>
@@ -7586,10 +8096,22 @@
       <c r="G24" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H24">
+        <v>1</v>
+      </c>
+      <c r="I24" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>419</v>
+        <v>447</v>
+      </c>
+      <c r="B25" t="s">
+        <v>448</v>
+      </c>
+      <c r="D25" t="s">
+        <v>426</v>
       </c>
       <c r="E25" t="s">
         <v>150</v>
@@ -7600,10 +8122,22 @@
       <c r="G25" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H25">
+        <v>1</v>
+      </c>
+      <c r="I25" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>420</v>
+        <v>449</v>
+      </c>
+      <c r="B26" t="s">
+        <v>450</v>
+      </c>
+      <c r="D26" t="s">
+        <v>426</v>
       </c>
       <c r="E26" t="s">
         <v>150</v>
@@ -7614,10 +8148,22 @@
       <c r="G26" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H26">
+        <v>1</v>
+      </c>
+      <c r="I26" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>421</v>
+        <v>451</v>
+      </c>
+      <c r="B27" t="s">
+        <v>452</v>
+      </c>
+      <c r="D27" t="s">
+        <v>426</v>
       </c>
       <c r="E27" t="s">
         <v>150</v>
@@ -7628,10 +8174,22 @@
       <c r="G27" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H27">
+        <v>1</v>
+      </c>
+      <c r="I27" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>422</v>
+        <v>453</v>
+      </c>
+      <c r="B28" t="s">
+        <v>454</v>
+      </c>
+      <c r="D28" t="s">
+        <v>426</v>
       </c>
       <c r="E28" t="s">
         <v>150</v>
@@ -7642,10 +8200,22 @@
       <c r="G28" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H28">
+        <v>1</v>
+      </c>
+      <c r="I28" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>423</v>
+        <v>455</v>
+      </c>
+      <c r="B29" t="s">
+        <v>456</v>
+      </c>
+      <c r="D29" t="s">
+        <v>426</v>
       </c>
       <c r="E29" t="s">
         <v>150</v>
@@ -7656,10 +8226,22 @@
       <c r="G29" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H29">
+        <v>1</v>
+      </c>
+      <c r="I29" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>424</v>
+        <v>457</v>
+      </c>
+      <c r="B30" t="s">
+        <v>458</v>
+      </c>
+      <c r="D30" t="s">
+        <v>426</v>
       </c>
       <c r="E30" t="s">
         <v>150</v>
@@ -7670,10 +8252,22 @@
       <c r="G30" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H30">
+        <v>1</v>
+      </c>
+      <c r="I30" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>425</v>
+        <v>459</v>
+      </c>
+      <c r="B31" t="s">
+        <v>460</v>
+      </c>
+      <c r="D31" t="s">
+        <v>426</v>
       </c>
       <c r="E31" t="s">
         <v>150</v>
@@ -7684,9 +8278,21 @@
       <c r="G31" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H31">
+        <v>1</v>
+      </c>
+      <c r="I31" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>461</v>
+      </c>
+      <c r="B32" t="s">
+        <v>462</v>
+      </c>
+      <c r="D32" t="s">
         <v>426</v>
       </c>
       <c r="E32" t="s">
@@ -7698,10 +8304,22 @@
       <c r="G32" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H32">
+        <v>1</v>
+      </c>
+      <c r="I32" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>427</v>
+        <v>463</v>
+      </c>
+      <c r="B33" t="s">
+        <v>464</v>
+      </c>
+      <c r="D33" t="s">
+        <v>426</v>
       </c>
       <c r="E33" t="s">
         <v>150</v>
@@ -7712,10 +8330,22 @@
       <c r="G33" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H33">
+        <v>1</v>
+      </c>
+      <c r="I33" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>428</v>
+        <v>465</v>
+      </c>
+      <c r="B34" t="s">
+        <v>466</v>
+      </c>
+      <c r="D34" t="s">
+        <v>426</v>
       </c>
       <c r="E34" t="s">
         <v>150</v>
@@ -7726,10 +8356,22 @@
       <c r="G34" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H34">
+        <v>1</v>
+      </c>
+      <c r="I34" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>429</v>
+        <v>467</v>
+      </c>
+      <c r="B35" t="s">
+        <v>468</v>
+      </c>
+      <c r="D35" t="s">
+        <v>426</v>
       </c>
       <c r="E35" t="s">
         <v>150</v>
@@ -7740,10 +8382,22 @@
       <c r="G35" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H35">
+        <v>1</v>
+      </c>
+      <c r="I35" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>430</v>
+        <v>469</v>
+      </c>
+      <c r="B36" t="s">
+        <v>470</v>
+      </c>
+      <c r="D36" t="s">
+        <v>410</v>
       </c>
       <c r="E36" t="s">
         <v>150</v>
@@ -7754,10 +8408,22 @@
       <c r="G36" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H36">
+        <v>1</v>
+      </c>
+      <c r="I36" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>431</v>
+        <v>471</v>
+      </c>
+      <c r="B37" t="s">
+        <v>472</v>
+      </c>
+      <c r="D37" t="s">
+        <v>410</v>
       </c>
       <c r="E37" t="s">
         <v>150</v>
@@ -7768,10 +8434,22 @@
       <c r="G37" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H37">
+        <v>1</v>
+      </c>
+      <c r="I37" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>432</v>
+        <v>473</v>
+      </c>
+      <c r="B38" t="s">
+        <v>474</v>
+      </c>
+      <c r="D38" t="s">
+        <v>426</v>
       </c>
       <c r="E38" t="s">
         <v>150</v>
@@ -7782,10 +8460,22 @@
       <c r="G38" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H38">
+        <v>1</v>
+      </c>
+      <c r="I38" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>433</v>
+        <v>475</v>
+      </c>
+      <c r="B39" t="s">
+        <v>476</v>
+      </c>
+      <c r="D39" t="s">
+        <v>426</v>
       </c>
       <c r="E39" t="s">
         <v>150</v>
@@ -7796,10 +8486,22 @@
       <c r="G39" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H39">
+        <v>1</v>
+      </c>
+      <c r="I39" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>434</v>
+        <v>477</v>
+      </c>
+      <c r="B40" t="s">
+        <v>478</v>
+      </c>
+      <c r="D40" t="s">
+        <v>410</v>
       </c>
       <c r="E40" t="s">
         <v>150</v>
@@ -7810,10 +8512,22 @@
       <c r="G40" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H40">
+        <v>1</v>
+      </c>
+      <c r="I40" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>435</v>
+        <v>479</v>
+      </c>
+      <c r="B41" t="s">
+        <v>480</v>
+      </c>
+      <c r="D41" t="s">
+        <v>426</v>
       </c>
       <c r="E41" t="s">
         <v>150</v>
@@ -7824,10 +8538,22 @@
       <c r="G41" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H41">
+        <v>1</v>
+      </c>
+      <c r="I41" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>436</v>
+        <v>481</v>
+      </c>
+      <c r="B42" t="s">
+        <v>482</v>
+      </c>
+      <c r="D42" t="s">
+        <v>410</v>
       </c>
       <c r="E42" t="s">
         <v>150</v>
@@ -7838,10 +8564,22 @@
       <c r="G42" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H42">
+        <v>1</v>
+      </c>
+      <c r="I42" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>437</v>
+        <v>483</v>
+      </c>
+      <c r="B43" t="s">
+        <v>484</v>
+      </c>
+      <c r="D43" t="s">
+        <v>426</v>
       </c>
       <c r="E43" t="s">
         <v>150</v>
@@ -7852,10 +8590,22 @@
       <c r="G43" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H43">
+        <v>1</v>
+      </c>
+      <c r="I43" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>438</v>
+        <v>485</v>
+      </c>
+      <c r="B44" t="s">
+        <v>486</v>
+      </c>
+      <c r="D44" t="s">
+        <v>410</v>
       </c>
       <c r="E44" t="s">
         <v>150</v>
@@ -7866,10 +8616,22 @@
       <c r="G44" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H44">
+        <v>1</v>
+      </c>
+      <c r="I44" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>439</v>
+        <v>487</v>
+      </c>
+      <c r="B45" t="s">
+        <v>488</v>
+      </c>
+      <c r="D45" t="s">
+        <v>426</v>
       </c>
       <c r="E45" t="s">
         <v>150</v>
@@ -7880,10 +8642,22 @@
       <c r="G45" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H45">
+        <v>1</v>
+      </c>
+      <c r="I45" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>440</v>
+        <v>489</v>
+      </c>
+      <c r="B46" t="s">
+        <v>490</v>
+      </c>
+      <c r="D46" t="s">
+        <v>426</v>
       </c>
       <c r="E46" t="s">
         <v>150</v>
@@ -7894,10 +8668,22 @@
       <c r="G46" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H46">
+        <v>1</v>
+      </c>
+      <c r="I46" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>441</v>
+        <v>491</v>
+      </c>
+      <c r="B47" t="s">
+        <v>492</v>
+      </c>
+      <c r="D47" t="s">
+        <v>410</v>
       </c>
       <c r="E47" t="s">
         <v>150</v>
@@ -7908,10 +8694,22 @@
       <c r="G47" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H47">
+        <v>1</v>
+      </c>
+      <c r="I47" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>442</v>
+        <v>493</v>
+      </c>
+      <c r="B48" t="s">
+        <v>494</v>
+      </c>
+      <c r="D48" t="s">
+        <v>410</v>
       </c>
       <c r="E48" t="s">
         <v>150</v>
@@ -7922,10 +8720,22 @@
       <c r="G48" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H48">
+        <v>1</v>
+      </c>
+      <c r="I48" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>443</v>
+        <v>495</v>
+      </c>
+      <c r="B49" t="s">
+        <v>496</v>
+      </c>
+      <c r="D49" t="s">
+        <v>426</v>
       </c>
       <c r="E49" t="s">
         <v>150</v>
@@ -7936,10 +8746,22 @@
       <c r="G49" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H49">
+        <v>1</v>
+      </c>
+      <c r="I49" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>444</v>
+        <v>497</v>
+      </c>
+      <c r="B50" t="s">
+        <v>498</v>
+      </c>
+      <c r="D50" t="s">
+        <v>426</v>
       </c>
       <c r="E50" t="s">
         <v>150</v>
@@ -7950,10 +8772,22 @@
       <c r="G50" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H50">
+        <v>1</v>
+      </c>
+      <c r="I50" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>445</v>
+        <v>499</v>
+      </c>
+      <c r="B51" t="s">
+        <v>500</v>
+      </c>
+      <c r="D51" t="s">
+        <v>426</v>
       </c>
       <c r="E51" t="s">
         <v>150</v>
@@ -7964,10 +8798,22 @@
       <c r="G51" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H51">
+        <v>1</v>
+      </c>
+      <c r="I51" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>446</v>
+        <v>501</v>
+      </c>
+      <c r="B52" t="s">
+        <v>502</v>
+      </c>
+      <c r="D52" t="s">
+        <v>426</v>
       </c>
       <c r="E52" t="s">
         <v>150</v>
@@ -7978,10 +8824,22 @@
       <c r="G52" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H52">
+        <v>1</v>
+      </c>
+      <c r="I52" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>447</v>
+        <v>503</v>
+      </c>
+      <c r="B53" t="s">
+        <v>504</v>
+      </c>
+      <c r="D53" t="s">
+        <v>426</v>
       </c>
       <c r="E53" t="s">
         <v>150</v>
@@ -7992,10 +8850,22 @@
       <c r="G53" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H53">
+        <v>1</v>
+      </c>
+      <c r="I53" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>448</v>
+        <v>505</v>
+      </c>
+      <c r="B54" t="s">
+        <v>506</v>
+      </c>
+      <c r="D54" t="s">
+        <v>426</v>
       </c>
       <c r="E54" t="s">
         <v>150</v>
@@ -8006,10 +8876,19 @@
       <c r="G54" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H54">
+        <v>1</v>
+      </c>
+      <c r="I54" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>449</v>
+        <v>507</v>
+      </c>
+      <c r="B55" t="s">
+        <v>535</v>
       </c>
       <c r="E55" t="s">
         <v>150</v>
@@ -8020,10 +8899,22 @@
       <c r="G55" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>450</v>
+      <c r="H55">
+        <v>0</v>
+      </c>
+      <c r="I55" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A56" s="6" t="s">
+        <v>508</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>539</v>
+      </c>
+      <c r="D56" t="s">
+        <v>410</v>
       </c>
       <c r="E56" t="s">
         <v>150</v>
@@ -8034,10 +8925,22 @@
       <c r="G56" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>451</v>
+      <c r="H56">
+        <v>0</v>
+      </c>
+      <c r="I56" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A57" s="6" t="s">
+        <v>509</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>534</v>
+      </c>
+      <c r="D57" t="s">
+        <v>410</v>
       </c>
       <c r="E57" t="s">
         <v>150</v>
@@ -8048,10 +8951,22 @@
       <c r="G57" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>452</v>
+      <c r="H57">
+        <v>0</v>
+      </c>
+      <c r="I57" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A58" s="6" t="s">
+        <v>510</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="D58" t="s">
+        <v>421</v>
       </c>
       <c r="E58" t="s">
         <v>150</v>
@@ -8062,10 +8977,22 @@
       <c r="G58" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H58">
+        <v>0</v>
+      </c>
+      <c r="I58" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>453</v>
+        <v>512</v>
+      </c>
+      <c r="B59" t="s">
+        <v>513</v>
+      </c>
+      <c r="D59" t="s">
+        <v>410</v>
       </c>
       <c r="E59" t="s">
         <v>150</v>
@@ -8076,10 +9003,22 @@
       <c r="G59" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>454</v>
+      <c r="H59">
+        <v>0</v>
+      </c>
+      <c r="I59" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A60" s="4" t="s">
+        <v>514</v>
+      </c>
+      <c r="B60" t="s">
+        <v>515</v>
+      </c>
+      <c r="D60" t="s">
+        <v>410</v>
       </c>
       <c r="E60" t="s">
         <v>150</v>
@@ -8090,10 +9029,22 @@
       <c r="G60" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>455</v>
+      <c r="H60">
+        <v>1</v>
+      </c>
+      <c r="I60" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A61" s="4" t="s">
+        <v>516</v>
+      </c>
+      <c r="B61" t="s">
+        <v>515</v>
+      </c>
+      <c r="D61" t="s">
+        <v>410</v>
       </c>
       <c r="E61" t="s">
         <v>150</v>
@@ -8104,10 +9055,22 @@
       <c r="G61" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H61">
+        <v>1</v>
+      </c>
+      <c r="I61" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>456</v>
+        <v>517</v>
+      </c>
+      <c r="B62" t="s">
+        <v>540</v>
+      </c>
+      <c r="D62" t="s">
+        <v>518</v>
       </c>
       <c r="E62" t="s">
         <v>150</v>
@@ -8118,10 +9081,22 @@
       <c r="G62" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H62">
+        <v>1</v>
+      </c>
+      <c r="I62" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>457</v>
+        <v>519</v>
+      </c>
+      <c r="B63" t="s">
+        <v>536</v>
+      </c>
+      <c r="D63" t="s">
+        <v>520</v>
       </c>
       <c r="E63" t="s">
         <v>150</v>
@@ -8132,10 +9107,22 @@
       <c r="G63" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H63">
+        <v>1</v>
+      </c>
+      <c r="I63" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>458</v>
+        <v>521</v>
+      </c>
+      <c r="B64" t="s">
+        <v>537</v>
+      </c>
+      <c r="D64" t="s">
+        <v>520</v>
       </c>
       <c r="E64" t="s">
         <v>150</v>
@@ -8146,10 +9133,22 @@
       <c r="G64" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H64">
+        <v>1</v>
+      </c>
+      <c r="I64" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>459</v>
+        <v>522</v>
+      </c>
+      <c r="B65" t="s">
+        <v>538</v>
+      </c>
+      <c r="D65" t="s">
+        <v>520</v>
       </c>
       <c r="E65" t="s">
         <v>150</v>
@@ -8160,10 +9159,22 @@
       <c r="G65" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H65">
+        <v>1</v>
+      </c>
+      <c r="I65" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>460</v>
+        <v>523</v>
+      </c>
+      <c r="B66" t="s">
+        <v>524</v>
+      </c>
+      <c r="D66" t="s">
+        <v>525</v>
       </c>
       <c r="E66" t="s">
         <v>150</v>
@@ -8174,10 +9185,22 @@
       <c r="G66" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H66">
+        <v>0</v>
+      </c>
+      <c r="I66" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>461</v>
+        <v>526</v>
+      </c>
+      <c r="B67" t="s">
+        <v>527</v>
+      </c>
+      <c r="D67" t="s">
+        <v>525</v>
       </c>
       <c r="E67" t="s">
         <v>150</v>
@@ -8188,10 +9211,19 @@
       <c r="G67" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>462</v>
+      <c r="H67">
+        <v>0</v>
+      </c>
+      <c r="I67" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A68" s="4" t="s">
+        <v>528</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>541</v>
       </c>
       <c r="E68" t="s">
         <v>150</v>
@@ -8202,10 +9234,19 @@
       <c r="G68" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>463</v>
+      <c r="H68">
+        <v>0</v>
+      </c>
+      <c r="I68" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A69" s="4" t="s">
+        <v>529</v>
+      </c>
+      <c r="B69" s="5" t="s">
+        <v>541</v>
       </c>
       <c r="E69" t="s">
         <v>150</v>
@@ -8216,10 +9257,19 @@
       <c r="G69" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>464</v>
+      <c r="H69">
+        <v>0</v>
+      </c>
+      <c r="I69" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A70" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="B70" s="5" t="s">
+        <v>541</v>
       </c>
       <c r="E70" t="s">
         <v>150</v>
@@ -8230,10 +9280,22 @@
       <c r="G70" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H70">
+        <v>0</v>
+      </c>
+      <c r="I70" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>465</v>
+        <v>531</v>
+      </c>
+      <c r="B71" t="s">
+        <v>532</v>
+      </c>
+      <c r="D71" t="s">
+        <v>533</v>
       </c>
       <c r="E71" t="s">
         <v>150</v>
@@ -8244,19 +9306,11 @@
       <c r="G71" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>466</v>
-      </c>
-      <c r="E72" t="s">
-        <v>150</v>
-      </c>
-      <c r="F72" t="s">
-        <v>150</v>
-      </c>
-      <c r="G72" t="s">
-        <v>197</v>
+      <c r="H71">
+        <v>1</v>
+      </c>
+      <c r="I71" t="s">
+        <v>400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
working on seabass data
</commit_message>
<xml_diff>
--- a/CMAP_variableMetadata_additions.xlsx
+++ b/CMAP_variableMetadata_additions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\GitHub_niskin\BWrepos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E14BE72-E1C8-4D5F-B170-33F1AF2DC8A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{063E24C3-D25B-4B98-BD50-985157914FC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="270" yWindow="165" windowWidth="35295" windowHeight="18930" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3450" yWindow="1050" windowWidth="28575" windowHeight="19110" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="notes" sheetId="4" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1961" uniqueCount="542">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1961" uniqueCount="545">
   <si>
     <t>Program</t>
   </si>
@@ -1652,7 +1652,16 @@
     <t>object_area_filled; Cross-sectional area of the target detected within the ROI determined by means specified in the image processing method or protocol document.</t>
   </si>
   <si>
-    <t>only net samples?</t>
+    <t>A life science identifier from a recognized taxonomic reference database (e.g., World Register of Marine Species, AlgaeBase) at the lowest level that matches the data provider's category, for a manual identification matched to scientificNameID. Generally, the ROI corresponds to an occurrence assigned to a single taxonomic name.</t>
+  </si>
+  <si>
+    <t>the fraction of the sample that was diluted (for example if you split the sample 4 times that is 1/16th of the total sample so 16 is the value used)</t>
+  </si>
+  <si>
+    <t>volume calculated from net flowmeter in L</t>
+  </si>
+  <si>
+    <t>Term to encompass the conversion from particles to particles/mL - in this case the volume (in mL) the net sample is diluted into before passing it through the FlowCam</t>
   </si>
 </sst>
 </file>
@@ -1683,24 +1692,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -1731,15 +1728,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -8907,10 +8902,10 @@
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A56" s="6" t="s">
+      <c r="A56" t="s">
         <v>508</v>
       </c>
-      <c r="B56" s="6" t="s">
+      <c r="B56" t="s">
         <v>539</v>
       </c>
       <c r="D56" t="s">
@@ -8933,10 +8928,10 @@
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A57" s="6" t="s">
+      <c r="A57" t="s">
         <v>509</v>
       </c>
-      <c r="B57" s="6" t="s">
+      <c r="B57" t="s">
         <v>534</v>
       </c>
       <c r="D57" t="s">
@@ -8959,10 +8954,10 @@
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A58" s="6" t="s">
+      <c r="A58" t="s">
         <v>510</v>
       </c>
-      <c r="B58" s="6" t="s">
+      <c r="B58" t="s">
         <v>511</v>
       </c>
       <c r="D58" t="s">
@@ -9041,7 +9036,7 @@
         <v>516</v>
       </c>
       <c r="B61" t="s">
-        <v>515</v>
+        <v>541</v>
       </c>
       <c r="D61" t="s">
         <v>410</v>
@@ -9222,8 +9217,8 @@
       <c r="A68" s="4" t="s">
         <v>528</v>
       </c>
-      <c r="B68" s="5" t="s">
-        <v>541</v>
+      <c r="B68" s="4" t="s">
+        <v>543</v>
       </c>
       <c r="E68" t="s">
         <v>150</v>
@@ -9245,8 +9240,8 @@
       <c r="A69" s="4" t="s">
         <v>529</v>
       </c>
-      <c r="B69" s="5" t="s">
-        <v>541</v>
+      <c r="B69" s="4" t="s">
+        <v>542</v>
       </c>
       <c r="E69" t="s">
         <v>150</v>
@@ -9268,8 +9263,8 @@
       <c r="A70" s="4" t="s">
         <v>530</v>
       </c>
-      <c r="B70" s="5" t="s">
-        <v>541</v>
+      <c r="B70" s="4" t="s">
+        <v>544</v>
       </c>
       <c r="E70" t="s">
         <v>150</v>

</xml_diff>